<commit_message>
Add building damage counts to results
</commit_message>
<xml_diff>
--- a/results/provinceResults.xlsx
+++ b/results/provinceResults.xlsx
@@ -5,27 +5,76 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshuadimasaka/Desktop/PhD/GitHub/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshuadimasaka/Desktop/PhD/GitHub/M78MaasimSaranganiEarthquakeRisk/results/expectedN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF76E569-F4D2-8447-BFEC-C7FEE461193B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8FB708F-ADBD-FA41-A7B0-7CAA17422666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4460" yWindow="3660" windowWidth="26840" windowHeight="15940" xr2:uid="{0A00CE89-1DC7-F742-A37A-8DFB79D5F69B}"/>
+    <workbookView xWindow="420" yWindow="11460" windowWidth="30000" windowHeight="8740" xr2:uid="{515E151D-AF91-9C42-A27E-A9EA3EAB23C3}"/>
   </bookViews>
   <sheets>
     <sheet name="adm2_risk" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>Province</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>adm1_psgc</t>
+  </si>
+  <si>
+    <t>adm2_psgc</t>
+  </si>
+  <si>
+    <t>adm2_en</t>
+  </si>
+  <si>
+    <t>Davao del Norte</t>
+  </si>
+  <si>
+    <t>Davao del Sur</t>
+  </si>
+  <si>
+    <t>Davao Oriental</t>
+  </si>
+  <si>
+    <t>Davao de Oro</t>
+  </si>
+  <si>
+    <t>Davao Occidental</t>
+  </si>
+  <si>
+    <t>Cotabato</t>
+  </si>
+  <si>
+    <t>South Cotabato</t>
+  </si>
+  <si>
+    <t>Sultan Kudarat</t>
+  </si>
+  <si>
+    <t>Sarangani</t>
+  </si>
+  <si>
+    <t>adm1_en</t>
   </si>
   <si>
     <t>Average Severe Damage Probability</t>
@@ -34,52 +83,29 @@
     <t>Average Collapse Damage Probability</t>
   </si>
   <si>
-    <t xml:space="preserve"> High-risk Building Count (Top 10%) </t>
+    <t>High-risk Building Count (Top 10%)</t>
   </si>
   <si>
     <t>High-Risk Concentration (Top 10%)</t>
   </si>
   <si>
-    <t>Region XII (SOCCSKSARGEN)</t>
-  </si>
-  <si>
-    <t>Sarangani</t>
-  </si>
-  <si>
-    <t>South Cotabato</t>
-  </si>
-  <si>
-    <t>Region XI (Davao Region)</t>
-  </si>
-  <si>
-    <t>Davao Occidental</t>
-  </si>
-  <si>
-    <t>Davao del Norte</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> -   </t>
-  </si>
-  <si>
-    <t>Davao del Sur</t>
-  </si>
-  <si>
-    <t>Davao Oriental</t>
-  </si>
-  <si>
-    <t>Davao de Oro</t>
-  </si>
-  <si>
-    <t>Cotabato</t>
-  </si>
-  <si>
-    <t>Sultan Kudarat</t>
+    <t>Expected number of damaged buildings</t>
+  </si>
+  <si>
+    <t>Expected number of severely damaged buildings</t>
+  </si>
+  <si>
+    <t>Expected number of collapsed buildings</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -513,8 +539,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -557,54 +585,72 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="44">
+    <cellStyle name="20% - Accent1" xfId="21" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="25" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="29" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="33" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="37" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="41" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="22" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="26" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="30" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="34" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="38" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="42" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="23" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="27" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="31" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="35" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="39" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="43" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="20" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="24" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="28" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="32" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="36" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="40" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="9" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="13" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="15" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Explanatory Text" xfId="18" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="8" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="4" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="5" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="6" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="7" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="11" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="14" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="10" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="17" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="12" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Title" xfId="3" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="19" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="16" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -617,6 +663,47 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="adm1_risk"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="A1" t="str">
+            <v>adm1_psgc</v>
+          </cell>
+          <cell r="B1" t="str">
+            <v>adm1_en</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="A2">
+            <v>1100000000</v>
+          </cell>
+          <cell r="B2" t="str">
+            <v>Region XI (Davao Region)</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3">
+            <v>1200000000</v>
+          </cell>
+          <cell r="B3" t="str">
+            <v>Region XII (SOCCSKSARGEN)</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -935,216 +1022,367 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C46DCDF9-3817-2E47-A8B1-5EE8971C9912}">
-  <dimension ref="A1:F10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{162DA48F-2F38-4B46-AFBC-4702ACEB7914}">
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.83203125" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" ht="85" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1100000000</v>
+      </c>
+      <c r="B2" t="str">
+        <f>VLOOKUP(A2, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XI (Davao Region)</v>
+      </c>
+      <c r="C2">
+        <v>1102300000</v>
+      </c>
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" s="5">
+        <v>1.10769967293239E-2</v>
+      </c>
+      <c r="F2" s="5">
+        <v>8.0863104495336002E-4</v>
+      </c>
+      <c r="G2" s="6">
+        <v>0</v>
+      </c>
+      <c r="H2" s="5">
+        <v>0</v>
+      </c>
+      <c r="I2" s="6">
+        <v>11306.8933090849</v>
+      </c>
+      <c r="J2" s="6">
+        <v>7991.2704021535701</v>
+      </c>
+      <c r="K2" s="6">
+        <v>367.859200446003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1100000000</v>
+      </c>
+      <c r="B3" t="str">
+        <f>VLOOKUP(A3, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XI (Davao Region)</v>
+      </c>
+      <c r="C3">
+        <v>1102400000</v>
+      </c>
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="E3" s="5">
+        <v>5.6777993574227199E-2</v>
+      </c>
+      <c r="F3" s="5">
+        <v>4.3889221520106098E-3</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6">
+        <v>38626.204337378796</v>
+      </c>
+      <c r="J3" s="6">
+        <v>30314.4176137348</v>
+      </c>
+      <c r="K3" s="6">
+        <v>1400.3690021198699</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1100000000</v>
+      </c>
+      <c r="B4" t="str">
+        <f>VLOOKUP(A4, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XI (Davao Region)</v>
+      </c>
+      <c r="C4">
+        <v>1102500000</v>
+      </c>
+      <c r="D4" t="s">
         <v>5</v>
       </c>
+      <c r="E4" s="5">
+        <v>7.4529974666883896E-3</v>
+      </c>
+      <c r="F4" s="5">
+        <v>5.3138038787758099E-4</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5">
+        <v>0</v>
+      </c>
+      <c r="I4" s="6">
+        <v>4056.8299917507602</v>
+      </c>
+      <c r="J4" s="6">
+        <v>2917.3384347859201</v>
+      </c>
+      <c r="K4" s="6">
+        <v>130.15524944595899</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1100000000</v>
+      </c>
+      <c r="B5" t="str">
+        <f>VLOOKUP(A5, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XI (Davao Region)</v>
+      </c>
+      <c r="C5">
+        <v>1108200000</v>
+      </c>
+      <c r="D5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E5" s="5">
+        <v>3.7682739462889E-3</v>
+      </c>
+      <c r="F5" s="5">
+        <v>2.5769066794973202E-4</v>
+      </c>
+      <c r="G5" s="6">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6">
+        <v>2887.5135286680502</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1957.18020084009</v>
+      </c>
+      <c r="K5" s="6">
+        <v>86.054767799141203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>1100000000</v>
+      </c>
+      <c r="B6" t="str">
+        <f>VLOOKUP(A6, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XI (Davao Region)</v>
+      </c>
+      <c r="C6">
+        <v>1108600000</v>
+      </c>
+      <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1">
-        <v>0.15640000000000001</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1.1900000000000001E-2</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="E6" s="5">
+        <v>7.0241063566323397E-2</v>
+      </c>
+      <c r="F6" s="5">
+        <v>4.0380321048346197E-3</v>
+      </c>
+      <c r="G6" s="6">
+        <v>697</v>
+      </c>
+      <c r="H6" s="5">
+        <v>7.8062875894587096E-3</v>
+      </c>
+      <c r="I6" s="6">
+        <v>12956.9754694894</v>
+      </c>
+      <c r="J6" s="6">
+        <v>10681.5721167226</v>
+      </c>
+      <c r="K6" s="6">
+        <v>360.54377254436798</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>1200000000</v>
+      </c>
+      <c r="B7" t="str">
+        <f>VLOOKUP(A7, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XII (SOCCSKSARGEN)</v>
+      </c>
+      <c r="C7">
+        <v>1204700000</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2.59353466755575E-2</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1.9798098244518301E-3</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6">
+        <v>31940.960659255499</v>
+      </c>
+      <c r="J7" s="6">
+        <v>23930.408629087298</v>
+      </c>
+      <c r="K7" s="6">
+        <v>1116.87803550731</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>1200000000</v>
+      </c>
+      <c r="B8" t="str">
+        <f>VLOOKUP(A8, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XII (SOCCSKSARGEN)</v>
+      </c>
+      <c r="C8">
+        <v>1206300000</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="5">
+        <v>0.12615863749183401</v>
+      </c>
+      <c r="F8" s="5">
+        <v>1.03670998944196E-2</v>
+      </c>
+      <c r="G8" s="6">
+        <v>44390</v>
+      </c>
+      <c r="H8" s="5">
+        <v>9.3982296013533098E-2</v>
+      </c>
+      <c r="I8" s="6">
+        <v>125804.50735768399</v>
+      </c>
+      <c r="J8" s="6">
+        <v>100953.04545699</v>
+      </c>
+      <c r="K8" s="6">
+        <v>4896.6197234319498</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>1200000000</v>
+      </c>
+      <c r="B9" t="str">
+        <f>VLOOKUP(A9, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XII (SOCCSKSARGEN)</v>
+      </c>
+      <c r="C9">
+        <v>1206500000</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="5">
+        <v>7.0994304455115995E-2</v>
+      </c>
+      <c r="F9" s="5">
+        <v>5.6900374845908503E-3</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6">
+        <v>52307.485243244497</v>
+      </c>
+      <c r="J9" s="6">
+        <v>40877.359924413096</v>
+      </c>
+      <c r="K9" s="6">
+        <v>1956.05849604031</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>1200000000</v>
+      </c>
+      <c r="B10" t="str">
+        <f>VLOOKUP(A10, [1]adm1_risk!$A:$B, 2, FALSE)</f>
+        <v>Region XII (SOCCSKSARGEN)</v>
+      </c>
+      <c r="C10">
+        <v>1208000000</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0.156422488146406</v>
+      </c>
+      <c r="F10" s="5">
+        <v>1.19349539626246E-2</v>
+      </c>
+      <c r="G10" s="6">
         <v>81064</v>
       </c>
-      <c r="F2" s="1">
-        <v>0.35460000000000003</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1">
-        <v>0.12620000000000001</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1.04E-2</v>
-      </c>
-      <c r="E3" s="2">
-        <v>44390</v>
-      </c>
-      <c r="F3" s="1">
-        <v>9.4E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1">
-        <v>7.0199999999999999E-2</v>
-      </c>
-      <c r="D4" s="1">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="E4">
-        <v>697</v>
-      </c>
-      <c r="F4" s="1">
-        <v>7.7999999999999996E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1.11E-2</v>
-      </c>
-      <c r="D5" s="1">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="1">
-        <v>5.6800000000000003E-2</v>
-      </c>
-      <c r="D6" s="1">
-        <v>4.4000000000000003E-3</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="1">
-        <v>7.4999999999999997E-3</v>
-      </c>
-      <c r="D7" s="1">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="1">
-        <v>3.8E-3</v>
-      </c>
-      <c r="D8" s="1">
-        <v>2.9999999999999997E-4</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="1">
-        <v>2.5899999999999999E-2</v>
-      </c>
-      <c r="D9" s="1">
-        <v>2E-3</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="1">
-        <v>7.0999999999999994E-2</v>
-      </c>
-      <c r="D10" s="1">
-        <v>5.7000000000000002E-3</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
+      <c r="H10" s="5">
+        <v>0.35460446886318697</v>
+      </c>
+      <c r="I10" s="6">
+        <v>73770.629667654895</v>
+      </c>
+      <c r="J10" s="6">
+        <v>61397.8089954631</v>
+      </c>
+      <c r="K10" s="6">
+        <v>2728.3782156718398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>